<commit_message>
Mejora de sistema vent
</commit_message>
<xml_diff>
--- a/Ventas/exports/reporte_semanal_2026-03-30_a_2026-04-05.xlsx
+++ b/Ventas/exports/reporte_semanal_2026-03-30_a_2026-04-05.xlsx
@@ -466,7 +466,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>288500</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6">
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>224080</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -486,7 +486,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>64420</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -530,15 +530,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -575,11 +575,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -589,71 +589,15 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>60000</v>
+        <v>116</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PAGADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Araceli</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>26600</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
           <t>ABONADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>22</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Jorge</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>201900</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
         </is>
       </c>
     </row>
@@ -668,13 +612,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -707,274 +651,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>10000</v>
+        <v>100</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B3" t="n">
-        <v>11</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>29000</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Efectivo</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>15000</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>efectivo</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B5" t="n">
-        <v>12</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>12400</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>transferencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B6" t="n">
-        <v>13</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>19000</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Efectivo</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>11</v>
-      </c>
-      <c r="B7" t="n">
-        <v>14</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>3800</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>12</v>
-      </c>
-      <c r="B8" t="n">
-        <v>15</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>13</v>
-      </c>
-      <c r="B9" t="n">
-        <v>15</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>8000</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>14</v>
-      </c>
-      <c r="B10" t="n">
-        <v>15</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>9280</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>15</v>
-      </c>
-      <c r="B11" t="n">
-        <v>19</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>3800</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>16</v>
-      </c>
-      <c r="B12" t="n">
-        <v>20</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Banco</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>17</v>
-      </c>
-      <c r="B13" t="n">
-        <v>21</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>3800</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>18</v>
-      </c>
-      <c r="B14" t="n">
-        <v>20</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>40000</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>f</t>
+          <t>w</t>
         </is>
       </c>
     </row>

</xml_diff>